<commit_message>
Add coordinator summary, agent briefs, open-model research and load estimate update
</commit_message>
<xml_diff>
--- a/docs/uoc-luong-tai.xlsx
+++ b/docs/uoc-luong-tai.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="GiaDinh" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="100">
   <si>
     <t xml:space="preserve">GIẢ ĐỊNH ĐẦU VÀO (chữ xanh = sửa được; chữ đen = công thức)</t>
   </si>
@@ -92,6 +92,9 @@
     <t xml:space="preserve">Output</t>
   </si>
   <si>
+    <t xml:space="preserve">Hỗ trợ prompt cache (1/0)</t>
+  </si>
+  <si>
     <t xml:space="preserve">small</t>
   </si>
   <si>
@@ -108,6 +111,12 @@
   </si>
   <si>
     <t xml:space="preserve">Opus (chưa kiểm giá)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">open</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DeepSeek V3.1 hoặc Qwen3 trên Bedrock (giá Sydney, CẦN KIỂM region và giá)</t>
   </si>
   <si>
     <t xml:space="preserve">5 CẤP TÁC VỤ</t>
@@ -770,7 +779,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J39"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
@@ -897,7 +906,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="40.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
         <v>19</v>
       </c>
@@ -910,13 +919,16 @@
       <c r="D14" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="E14" s="4" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C15" s="2" t="n">
         <v>1</v>
@@ -924,13 +936,16 @@
       <c r="D15" s="2" t="n">
         <v>5</v>
       </c>
+      <c r="E15" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C16" s="2" t="n">
         <v>3</v>
@@ -938,13 +953,16 @@
       <c r="D16" s="2" t="n">
         <v>15</v>
       </c>
+      <c r="E16" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>5</v>
@@ -952,47 +970,67 @@
       <c r="D17" s="2" t="n">
         <v>25</v>
       </c>
+      <c r="E17" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="27.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>19</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>0.45</v>
@@ -1004,7 +1042,7 @@
         <v>400</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>0</v>
@@ -1019,12 +1057,12 @@
         <v>0</v>
       </c>
       <c r="J21" s="0" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>0.2</v>
@@ -1036,7 +1074,7 @@
         <v>2000</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F22" s="2" t="n">
         <v>0.5</v>
@@ -1051,12 +1089,12 @@
         <v>0</v>
       </c>
       <c r="J22" s="0" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>0.15</v>
@@ -1068,7 +1106,7 @@
         <v>1500</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F23" s="2" t="n">
         <v>0.9</v>
@@ -1083,12 +1121,12 @@
         <v>0</v>
       </c>
       <c r="J23" s="0" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>0.15</v>
@@ -1100,7 +1138,7 @@
         <v>4000</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F24" s="2" t="n">
         <v>0.3</v>
@@ -1115,12 +1153,12 @@
         <v>0</v>
       </c>
       <c r="J24" s="0" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>0.05</v>
@@ -1132,7 +1170,7 @@
         <v>1500</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F25" s="2" t="n">
         <v>0.3</v>
@@ -1147,12 +1185,12 @@
         <v>2</v>
       </c>
       <c r="J25" s="0" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B26" s="0" t="n">
         <f aca="false">SUM(B21:B25)</f>
@@ -1161,23 +1199,23 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>2</v>
       </c>
       <c r="C29" s="0" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>10</v>
@@ -1188,7 +1226,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>500000</v>
@@ -1199,7 +1237,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>8</v>
@@ -1210,7 +1248,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>1024</v>
@@ -1221,7 +1259,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>4</v>
@@ -1229,29 +1267,29 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>20</v>
       </c>
       <c r="C35" s="0" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>12</v>
       </c>
       <c r="C36" s="0" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>50</v>
@@ -1262,7 +1300,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>500</v>
@@ -1273,7 +1311,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>10</v>
@@ -1299,7 +1337,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K32"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="2" style="0" width="18"/>
@@ -1312,47 +1350,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="27.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1373,11 +1411,11 @@
         <v>198</v>
       </c>
       <c r="E4" s="6" t="n">
-        <f aca="false">C4*(GiaDinh!$B$10*GiaDinh!$B$11+(1-GiaDinh!$B$10))*VLOOKUP(GiaDinh!E21,GiaDinh!$A$15:$D$17,3,FALSE())</f>
+        <f aca="false">C4*(1-GiaDinh!$B$10*VLOOKUP(GiaDinh!E21,GiaDinh!$A$15:$E$18,5,FALSE())*(1-GiaDinh!$B$11))*VLOOKUP(GiaDinh!E21,GiaDinh!$A$15:$E$18,3,FALSE())</f>
         <v>816.75</v>
       </c>
       <c r="F4" s="6" t="n">
-        <f aca="false">D4*VLOOKUP(GiaDinh!E21,GiaDinh!$A$15:$D$17,4,FALSE())</f>
+        <f aca="false">D4*VLOOKUP(GiaDinh!E21,GiaDinh!$A$15:$E$18,4,FALSE())</f>
         <v>990</v>
       </c>
       <c r="G4" s="6" t="n">
@@ -1419,11 +1457,11 @@
         <v>440</v>
       </c>
       <c r="E5" s="6" t="n">
-        <f aca="false">C5*(GiaDinh!$B$10*GiaDinh!$B$11+(1-GiaDinh!$B$10))*VLOOKUP(GiaDinh!E22,GiaDinh!$A$15:$D$17,3,FALSE())</f>
+        <f aca="false">C5*(1-GiaDinh!$B$10*VLOOKUP(GiaDinh!E22,GiaDinh!$A$15:$E$18,5,FALSE())*(1-GiaDinh!$B$11))*VLOOKUP(GiaDinh!E22,GiaDinh!$A$15:$E$18,3,FALSE())</f>
         <v>2178</v>
       </c>
       <c r="F5" s="6" t="n">
-        <f aca="false">D5*VLOOKUP(GiaDinh!E22,GiaDinh!$A$15:$D$17,4,FALSE())</f>
+        <f aca="false">D5*VLOOKUP(GiaDinh!E22,GiaDinh!$A$15:$E$18,4,FALSE())</f>
         <v>6600</v>
       </c>
       <c r="G5" s="6" t="n">
@@ -1465,11 +1503,11 @@
         <v>247.5</v>
       </c>
       <c r="E6" s="6" t="n">
-        <f aca="false">C6*(GiaDinh!$B$10*GiaDinh!$B$11+(1-GiaDinh!$B$10))*VLOOKUP(GiaDinh!E23,GiaDinh!$A$15:$D$17,3,FALSE())</f>
+        <f aca="false">C6*(1-GiaDinh!$B$10*VLOOKUP(GiaDinh!E23,GiaDinh!$A$15:$E$18,5,FALSE())*(1-GiaDinh!$B$11))*VLOOKUP(GiaDinh!E23,GiaDinh!$A$15:$E$18,3,FALSE())</f>
         <v>2722.5</v>
       </c>
       <c r="F6" s="6" t="n">
-        <f aca="false">D6*VLOOKUP(GiaDinh!E23,GiaDinh!$A$15:$D$17,4,FALSE())</f>
+        <f aca="false">D6*VLOOKUP(GiaDinh!E23,GiaDinh!$A$15:$E$18,4,FALSE())</f>
         <v>3712.5</v>
       </c>
       <c r="G6" s="6" t="n">
@@ -1511,11 +1549,11 @@
         <v>660</v>
       </c>
       <c r="E7" s="6" t="n">
-        <f aca="false">C7*(GiaDinh!$B$10*GiaDinh!$B$11+(1-GiaDinh!$B$10))*VLOOKUP(GiaDinh!E24,GiaDinh!$A$15:$D$17,3,FALSE())</f>
+        <f aca="false">C7*(1-GiaDinh!$B$10*VLOOKUP(GiaDinh!E24,GiaDinh!$A$15:$E$18,5,FALSE())*(1-GiaDinh!$B$11))*VLOOKUP(GiaDinh!E24,GiaDinh!$A$15:$E$18,3,FALSE())</f>
         <v>10890</v>
       </c>
       <c r="F7" s="6" t="n">
-        <f aca="false">D7*VLOOKUP(GiaDinh!E24,GiaDinh!$A$15:$D$17,4,FALSE())</f>
+        <f aca="false">D7*VLOOKUP(GiaDinh!E24,GiaDinh!$A$15:$E$18,4,FALSE())</f>
         <v>9900</v>
       </c>
       <c r="G7" s="6" t="n">
@@ -1557,11 +1595,11 @@
         <v>82.5</v>
       </c>
       <c r="E8" s="6" t="n">
-        <f aca="false">C8*(GiaDinh!$B$10*GiaDinh!$B$11+(1-GiaDinh!$B$10))*VLOOKUP(GiaDinh!E25,GiaDinh!$A$15:$D$17,3,FALSE())</f>
+        <f aca="false">C8*(1-GiaDinh!$B$10*VLOOKUP(GiaDinh!E25,GiaDinh!$A$15:$E$18,5,FALSE())*(1-GiaDinh!$B$11))*VLOOKUP(GiaDinh!E25,GiaDinh!$A$15:$E$18,3,FALSE())</f>
         <v>907.5</v>
       </c>
       <c r="F8" s="6" t="n">
-        <f aca="false">D8*VLOOKUP(GiaDinh!E25,GiaDinh!$A$15:$D$17,4,FALSE())</f>
+        <f aca="false">D8*VLOOKUP(GiaDinh!E25,GiaDinh!$A$15:$E$18,4,FALSE())</f>
         <v>2062.5</v>
       </c>
       <c r="G8" s="6" t="n">
@@ -1587,7 +1625,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B9" s="7" t="n">
         <f aca="false">SUM(B4:B8)</f>
@@ -1632,7 +1670,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">K9/GiaDinh!B3</f>
@@ -1662,7 +1700,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -1677,7 +1715,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">GiaDinh!B3*GiaDinh!B4</f>
@@ -1695,7 +1733,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B14" s="6" t="n">
         <f aca="false">B13*GiaDinh!B5</f>
@@ -1713,7 +1751,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B15" s="6" t="n">
         <f aca="false">B13*GiaDinh!B7</f>
@@ -1731,7 +1769,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">B15/3600</f>
@@ -1749,7 +1787,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">B16*GiaDinh!B8</f>
@@ -1767,7 +1805,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B18" s="6" t="n">
         <f aca="false">GiaDinh!B3*GiaDinh!B9</f>
@@ -1785,7 +1823,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">C9*1000000/GiaDinh!B5*GiaDinh!B7/3600*GiaDinh!B8</f>
@@ -1803,7 +1841,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">D9*1000000/GiaDinh!B5*GiaDinh!B7/3600*GiaDinh!B8</f>
@@ -1821,7 +1859,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B21" s="8" t="n">
         <f aca="false">H9/GiaDinh!B5*GiaDinh!B7*GiaDinh!B8</f>
@@ -1851,7 +1889,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -1866,7 +1904,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B24" s="6" t="n">
         <f aca="false">GiaDinh!B3*GiaDinh!B29/1024</f>
@@ -1884,7 +1922,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B25" s="6" t="n">
         <f aca="false">GiaDinh!B3*GiaDinh!B30/1024</f>
@@ -1902,7 +1940,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="B26" s="6" t="n">
         <f aca="false">GiaDinh!B31*GiaDinh!B32</f>
@@ -1920,7 +1958,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B27" s="6" t="n">
         <f aca="false">B26*GiaDinh!B33*GiaDinh!B34/1000000000</f>
@@ -1938,7 +1976,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B28" s="6" t="n">
         <f aca="false">B14*GiaDinh!B35/1000000</f>
@@ -1956,7 +1994,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B29" s="6" t="n">
         <f aca="false">B28*GiaDinh!B36</f>
@@ -1974,7 +2012,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B30" s="6" t="n">
         <f aca="false">J9*GiaDinh!B38/1000000</f>
@@ -1992,7 +2030,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B31" s="6" t="n">
         <f aca="false">I9*GiaDinh!B37/1000000</f>
@@ -2010,7 +2048,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B32" s="6" t="n">
         <f aca="false">B14*GiaDinh!B39/1000000*12</f>

</xml_diff>

<commit_message>
Finalise decisions, regenerate deck and quote workbook (total 18871.95)
</commit_message>
<xml_diff>
--- a/docs/uoc-luong-tai.xlsx
+++ b/docs/uoc-luong-tai.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="GiaDinh" sheetId="1" state="visible" r:id="rId3"/>
@@ -176,7 +176,7 @@
     <t xml:space="preserve">Cấp 5 Thiết kế</t>
   </si>
   <si>
-    <t xml:space="preserve">Có sinh ảnh</t>
+    <t xml:space="preserve">1 ảnh nháp, trung bình 1,1 ảnh/request</t>
   </si>
   <si>
     <t xml:space="preserve">Tổng tỉ lệ (phải bằng 1)</t>
@@ -1182,7 +1182,7 @@
         <v>1</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>2</v>
+        <v>1.1</v>
       </c>
       <c r="J25" s="0" t="s">
         <v>51</v>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="J8" s="6" t="n">
         <f aca="false">B8*GiaDinh!I25</f>
-        <v>110000</v>
+        <v>60500</v>
       </c>
       <c r="K8" s="6" t="n">
         <f aca="false">E8+F8</f>
@@ -1661,7 +1661,7 @@
       </c>
       <c r="J9" s="7" t="n">
         <f aca="false">SUM(J4:J8)</f>
-        <v>110000</v>
+        <v>60500</v>
       </c>
       <c r="K9" s="7" t="n">
         <f aca="false">SUM(K4:K8)</f>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B30" s="6" t="n">
         <f aca="false">J9*GiaDinh!B38/1000000</f>
-        <v>55</v>
+        <v>30.25</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>

</xml_diff>